<commit_message>
path changes to point to result folder
</commit_message>
<xml_diff>
--- a/results/model_results_bean.xlsx
+++ b/results/model_results_bean.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,11 @@
           <t>Time (s)</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Data_norm</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -481,6 +486,7 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -492,23 +498,24 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9242284982174688</v>
+        <v>0.9246878038405445</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9250448034975397</v>
+        <v>0.9254856636012668</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9242284982174688</v>
+        <v>0.9246878038405445</v>
       </c>
       <c r="F3" t="n">
-        <v>0.924388462098727</v>
+        <v>0.9248435995994724</v>
       </c>
       <c r="G3" t="n">
         <v>100</v>
       </c>
       <c r="H3" t="n">
-        <v>11.09081888198853</v>
-      </c>
+        <v>3.163018941879272</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -533,370 +540,385 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Input_hpt</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0.1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2640522031815481</v>
+        <v>0.2464193903782593</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6851951204897102</v>
+        <v>0.8143031255761337</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2640522031815481</v>
+        <v>0.2464193903782593</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1109084246609548</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.9901168346405029</v>
-      </c>
+        <v>0.09743512725033115</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Input_hpt</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="C6" t="n">
-        <v>0.2475211164157179</v>
+        <v>0.2640522031815481</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8143700989393187</v>
+        <v>0.6851951204897102</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2475211164157179</v>
+        <v>0.2640522031815481</v>
       </c>
       <c r="F6" t="n">
-        <v>0.09966969337187191</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+        <v>0.1109084246609548</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.3131580352783203</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Input_hpt</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2638687172527413</v>
+        <v>0.2475211164157179</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2425770580854837</v>
+        <v>0.8143700989393187</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2638687172527413</v>
+        <v>0.2475211164157179</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1597879656845585</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1.126983642578125</v>
-      </c>
+        <v>0.09966969337187191</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Input_hpt</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.5875872199779655</v>
+        <v>0.2638687172527413</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6342684410431411</v>
+        <v>0.2425770580854837</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5875872199779655</v>
+        <v>0.2638687172527413</v>
       </c>
       <c r="F8" t="n">
-        <v>0.5454336561368643</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+        <v>0.1597879656845585</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.3037450313568115</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Input_hpt</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>0.457569005563658</v>
+        <v>0.5875872199779655</v>
       </c>
       <c r="D9" t="n">
-        <v>0.4331267451365911</v>
+        <v>0.6342684410431411</v>
       </c>
       <c r="E9" t="n">
-        <v>0.457569005563658</v>
+        <v>0.5875872199779655</v>
       </c>
       <c r="F9" t="n">
-        <v>0.435187715561223</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" t="n">
-        <v>1.519360542297363</v>
-      </c>
+        <v>0.5454336561368643</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Input_hpt</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8398824825560044</v>
+        <v>0.457569005563658</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8557032386130576</v>
+        <v>0.4331267451365911</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8398824825560044</v>
+        <v>0.457569005563658</v>
       </c>
       <c r="F10" t="n">
-        <v>0.8361008605573937</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+        <v>0.435187715561223</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.3848278522491455</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Input_hpt</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.6362026008750608</v>
+        <v>0.8398824825560044</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6319002127889755</v>
+        <v>0.8557032386130576</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6362026008750608</v>
+        <v>0.8398824825560044</v>
       </c>
       <c r="F11" t="n">
-        <v>0.6321107078831846</v>
-      </c>
-      <c r="G11" t="n">
-        <v>100</v>
-      </c>
-      <c r="H11" t="n">
-        <v>2.285573244094849</v>
-      </c>
+        <v>0.8361008605573937</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Input_hpt</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9166360631656262</v>
+        <v>0.6362026008750608</v>
       </c>
       <c r="D12" t="n">
-        <v>0.917664304733454</v>
+        <v>0.6319002127889755</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9166360631656262</v>
+        <v>0.6362026008750608</v>
       </c>
       <c r="F12" t="n">
-        <v>0.9168047279409691</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+        <v>0.6321107078831846</v>
+      </c>
+      <c r="G12" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.5006780624389648</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Input_hpt</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>30</v>
       </c>
       <c r="C13" t="n">
-        <v>0.8483640718684168</v>
+        <v>0.9166360631656262</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8490751939066769</v>
+        <v>0.917664304733454</v>
       </c>
       <c r="E13" t="n">
-        <v>0.8483640718684168</v>
+        <v>0.9166360631656262</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8480880058376593</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" t="n">
-        <v>3.221936225891113</v>
-      </c>
+        <v>0.9168047279409691</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Input_hpt</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C14" t="n">
-        <v>0.9236136614028645</v>
+        <v>0.8483640718684168</v>
       </c>
       <c r="D14" t="n">
-        <v>0.924783804348453</v>
+        <v>0.8490751939066769</v>
       </c>
       <c r="E14" t="n">
-        <v>0.9236136614028645</v>
+        <v>0.8483640718684168</v>
       </c>
       <c r="F14" t="n">
-        <v>0.923896521417948</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+        <v>0.8480880058376593</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.6757259368896484</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Input_hpt</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>50</v>
       </c>
       <c r="C15" t="n">
-        <v>0.8923590011073299</v>
+        <v>0.9236136614028645</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8931292811016809</v>
+        <v>0.924783804348453</v>
       </c>
       <c r="E15" t="n">
-        <v>0.8923590011073299</v>
+        <v>0.9236136614028645</v>
       </c>
       <c r="F15" t="n">
-        <v>0.8924761032092201</v>
-      </c>
-      <c r="G15" t="n">
-        <v>10</v>
-      </c>
-      <c r="H15" t="n">
-        <v>3.376485347747803</v>
-      </c>
+        <v>0.923896521417948</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Input_hpt</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C16" t="n">
-        <v>0.9254498714652957</v>
+        <v>0.8923590011073299</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9263203338154221</v>
+        <v>0.8931292811016809</v>
       </c>
       <c r="E16" t="n">
-        <v>0.9254498714652957</v>
+        <v>0.8923590011073299</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9257356025609044</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+        <v>0.8924761032092201</v>
+      </c>
+      <c r="G16" t="n">
+        <v>10</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.6333959102630615</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Input_hpt</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>100</v>
       </c>
       <c r="C17" t="n">
-        <v>0.9130237873386269</v>
+        <v>0.9254498714652957</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9137150503572755</v>
+        <v>0.9263203338154221</v>
       </c>
       <c r="E17" t="n">
-        <v>0.9130237873386269</v>
+        <v>0.9254498714652957</v>
       </c>
       <c r="F17" t="n">
-        <v>0.9131404216655179</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" t="n">
-        <v>3.369741916656494</v>
-      </c>
+        <v>0.9257356025609044</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>Input_hpt</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="C18" t="n">
-        <v>0.9265515975027543</v>
+        <v>0.9130237873386269</v>
       </c>
       <c r="D18" t="n">
-        <v>0.9277901329477568</v>
+        <v>0.9137150503572755</v>
       </c>
       <c r="E18" t="n">
-        <v>0.9265515975027543</v>
+        <v>0.9130237873386269</v>
       </c>
       <c r="F18" t="n">
-        <v>0.9269362635447583</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+        <v>0.9131404216655179</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.6637859344482422</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -905,7 +927,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="C19" t="n">
         <v>0.9265515975027543</v>
@@ -921,6 +943,7 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -929,7 +952,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C20" t="n">
         <v>0.9265515975027543</v>
@@ -945,6 +968,7 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -953,7 +977,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
         <v>0.9265515975027543</v>
@@ -969,6 +993,7 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -977,7 +1002,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C22" t="n">
         <v>0.9265515975027543</v>
@@ -993,6 +1018,7 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1001,7 +1027,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C23" t="n">
         <v>0.9265515975027543</v>
@@ -1017,6 +1043,7 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1025,7 +1052,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C24" t="n">
         <v>0.9265515975027543</v>
@@ -1041,6 +1068,235 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>100</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.9265515975027543</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.9277901329477568</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.9265515975027543</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.9269362635447583</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.08960705104663974</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.07283145075144473</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.08960705104663974</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.07444035707153802</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>0.04343724250793457</v>
+      </c>
+      <c r="I26" t="n">
+        <v>18.68894470696321</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.3371281674623577</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.2567094915012275</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.3371281674623577</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.283979608935134</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0.0404658317565918</v>
+      </c>
+      <c r="I27" t="n">
+        <v>18.68894470696321</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.6973925817113478</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.7012349547071757</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.6973925817113478</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.69462977310209</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0.05654716491699219</v>
+      </c>
+      <c r="I28" t="n">
+        <v>18.68894470696321</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>10</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.8057289753947852</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.8160513335758859</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.8057289753947852</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.8082760304973603</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>0.06341695785522461</v>
+      </c>
+      <c r="I29" t="n">
+        <v>18.68894470696321</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>30</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.7958134410576569</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.842601799574785</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.7958134410576569</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.8041308329429669</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>0.07846784591674805</v>
+      </c>
+      <c r="I30" t="n">
+        <v>18.68894470696321</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>50</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.9045170767535806</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.9077486982519526</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.9045170767535806</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.9054878856586722</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>0.08301305770874023</v>
+      </c>
+      <c r="I31" t="n">
+        <v>18.68894470696321</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>100</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.9177377892030848</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.9197931529053442</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.9177377892030848</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.9183336746698749</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>0.08047103881835938</v>
+      </c>
+      <c r="I32" t="n">
+        <v>18.68894470696321</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>